<commit_message>
Fix locale-specific artifacts in spreadsheet templates
</commit_message>
<xml_diff>
--- a/new/be-BY/new.xlsx
+++ b/new/be-BY/new.xlsx
@@ -7,7 +7,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11985"/>
   </bookViews>
   <sheets>
-    <sheet name="Аркуш1" sheetId="1" r:id="rId1"/>
+    <sheet name="Лiст1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -53,7 +53,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Звычайны" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>

</xml_diff>